<commit_message>
vault backup: 2026-04-28 21:21:07
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/MNST/MNST_model.xlsx
+++ b/Knowledge/Model Outputs/MNST/MNST_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodin\Desktop\Brain\Knowledge\Model Outputs\MNST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4494808D-52CD-41C0-905D-FD3F44160813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A5A73C-4B0C-4130-BC1E-E73248AE8B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4810,83 +4810,83 @@
       </c>
       <c r="Z22" s="11">
         <f>'CF DRIVERS'!Z22</f>
-        <v>0</v>
+        <v>4815.9971645233672</v>
       </c>
       <c r="AA22" s="11">
         <f>'CF DRIVERS'!AA22</f>
-        <v>0</v>
+        <v>29114.825015548769</v>
       </c>
       <c r="AB22" s="11">
         <f>'CF DRIVERS'!AB22</f>
-        <v>0</v>
+        <v>9690.2162765632165</v>
       </c>
       <c r="AC22" s="11">
         <f>'CF DRIVERS'!AC22</f>
-        <v>0</v>
+        <v>-7485.8246022026797</v>
       </c>
       <c r="AD22" s="11">
         <f>'CF DRIVERS'!AD22</f>
-        <v>0</v>
+        <v>5663.8592644697201</v>
       </c>
       <c r="AE22" s="11">
         <f>'CF DRIVERS'!AE22</f>
-        <v>0</v>
+        <v>34240.525017844666</v>
       </c>
       <c r="AF22" s="11">
         <f>'CF DRIVERS'!AF22</f>
-        <v>0</v>
+        <v>11396.190520423574</v>
       </c>
       <c r="AG22" s="11">
         <f>'CF DRIVERS'!AG22</f>
-        <v>0</v>
+        <v>-8803.7130373969849</v>
       </c>
       <c r="AH22" s="11">
         <f>'CF DRIVERS'!AH22</f>
-        <v>0</v>
+        <v>6660.9885080558233</v>
       </c>
       <c r="AI22" s="11">
         <f>'CF DRIVERS'!AI22</f>
-        <v>0</v>
+        <v>40268.610677602192</v>
       </c>
       <c r="AJ22" s="11">
         <f>'CF DRIVERS'!AJ22</f>
-        <v>0</v>
+        <v>13402.503584146376</v>
       </c>
       <c r="AK22" s="11">
         <f>'CF DRIVERS'!AK22</f>
-        <v>0</v>
+        <v>-10353.617318528588</v>
       </c>
       <c r="AL22" s="11">
         <f>'CF DRIVERS'!AL22</f>
-        <v>0</v>
+        <v>7833.6635556578985</v>
       </c>
       <c r="AM22" s="11">
         <f>'CF DRIVERS'!AM22</f>
-        <v>0</v>
+        <v>47357.948076415589</v>
       </c>
       <c r="AN22" s="11">
         <f>'CF DRIVERS'!AN22</f>
-        <v>0</v>
+        <v>15762.030478618326</v>
       </c>
       <c r="AO22" s="11">
         <f>'CF DRIVERS'!AO22</f>
-        <v>0</v>
+        <v>-12176.384114654415</v>
       </c>
       <c r="AP22" s="11">
         <f>'CF DRIVERS'!AP22</f>
-        <v>0</v>
+        <v>9212.7894574545571</v>
       </c>
       <c r="AQ22" s="11">
         <f>'CF DRIVERS'!AQ22</f>
-        <v>0</v>
+        <v>55695.371860840714</v>
       </c>
       <c r="AR22" s="11">
         <f>'CF DRIVERS'!AR22</f>
-        <v>0</v>
+        <v>18536.954924061356</v>
       </c>
       <c r="AS22" s="11">
         <f>'CF DRIVERS'!AS22</f>
-        <v>0</v>
+        <v>-14320.051200103422</v>
       </c>
     </row>
     <row r="23" spans="1:45" x14ac:dyDescent="0.25">
@@ -5172,83 +5172,83 @@
       </c>
       <c r="Z24" s="7">
         <f t="shared" ref="Z24:AS24" si="0">SUM(Z2:Z23)</f>
-        <v>507366.04979337979</v>
+        <v>512182.04695790313</v>
       </c>
       <c r="AA24" s="7">
         <f t="shared" si="0"/>
-        <v>433233.00936874747</v>
+        <v>462347.83438429626</v>
       </c>
       <c r="AB24" s="7">
         <f t="shared" si="0"/>
-        <v>572854.57586070639</v>
+        <v>582544.79213726963</v>
       </c>
       <c r="AC24" s="7">
         <f t="shared" si="0"/>
-        <v>657177.62129324151</v>
+        <v>649691.79669103888</v>
       </c>
       <c r="AD24" s="7">
         <f t="shared" si="0"/>
-        <v>592457.61741658114</v>
+        <v>598121.47668105084</v>
       </c>
       <c r="AE24" s="7">
         <f t="shared" si="0"/>
-        <v>505273.36595867545</v>
+        <v>539513.89097652014</v>
       </c>
       <c r="AF24" s="7">
         <f t="shared" si="0"/>
-        <v>669475.47735537635</v>
+        <v>680871.66787579993</v>
       </c>
       <c r="AG24" s="7">
         <f t="shared" si="0"/>
-        <v>768643.69647301291</v>
+        <v>759839.9834356159</v>
       </c>
       <c r="AH24" s="7">
         <f t="shared" si="0"/>
-        <v>692529.65798195684</v>
+        <v>699190.64649001264</v>
       </c>
       <c r="AI24" s="7">
         <f t="shared" si="0"/>
-        <v>589996.51407289389</v>
+        <v>630265.12475049612</v>
       </c>
       <c r="AJ24" s="7">
         <f t="shared" si="0"/>
-        <v>783106.60490321869</v>
+        <v>796509.10848736507</v>
       </c>
       <c r="AK24" s="7">
         <f t="shared" si="0"/>
-        <v>899733.50840887695</v>
+        <v>889379.89109034836</v>
       </c>
       <c r="AL24" s="7">
         <f t="shared" si="0"/>
-        <v>810219.50178955751</v>
+        <v>818053.16534521547</v>
       </c>
       <c r="AM24" s="7">
         <f t="shared" si="0"/>
-        <v>689635.27443110279</v>
+        <v>736993.22250751837</v>
       </c>
       <c r="AN24" s="7">
         <f t="shared" si="0"/>
-        <v>916742.62928357895</v>
+        <v>932504.65976219729</v>
       </c>
       <c r="AO24" s="7">
         <f t="shared" si="0"/>
-        <v>1053901.8395864605</v>
+        <v>1041725.4554718061</v>
       </c>
       <c r="AP24" s="7">
         <f t="shared" si="0"/>
-        <v>948628.78431446548</v>
+        <v>957841.57377192006</v>
       </c>
       <c r="AQ24" s="7">
         <f t="shared" si="0"/>
-        <v>806815.55852933368</v>
+        <v>862510.93039017438</v>
       </c>
       <c r="AR24" s="7">
         <f t="shared" si="0"/>
-        <v>1073905.4366725073</v>
+        <v>1092442.3915965687</v>
       </c>
       <c r="AS24" s="7">
         <f t="shared" si="0"/>
-        <v>1235211.6911080228</v>
+        <v>1220891.6399079193</v>
       </c>
     </row>
     <row r="25" spans="1:45" x14ac:dyDescent="0.25">
@@ -8587,83 +8587,83 @@
       </c>
       <c r="Z43" s="7">
         <f t="shared" ref="Z43:AS43" si="3">Z24+Z33+Z41+Z42</f>
-        <v>492210.49508407683</v>
+        <v>497026.49224860017</v>
       </c>
       <c r="AA43" s="7">
         <f t="shared" si="3"/>
-        <v>356388.98789241223</v>
+        <v>385503.81290796102</v>
       </c>
       <c r="AB43" s="7">
         <f t="shared" si="3"/>
-        <v>540799.75702492963</v>
+        <v>550489.97330149286</v>
       </c>
       <c r="AC43" s="7">
         <f t="shared" si="3"/>
-        <v>666930.94479695905</v>
+        <v>659445.12019475643</v>
       </c>
       <c r="AD43" s="7">
         <f t="shared" si="3"/>
-        <v>570212.55911054707</v>
+        <v>575876.41837501677</v>
       </c>
       <c r="AE43" s="7">
         <f t="shared" si="3"/>
-        <v>410479.51202975848</v>
+        <v>444720.03704760317</v>
       </c>
       <c r="AF43" s="7">
         <f t="shared" si="3"/>
-        <v>627356.01912433258</v>
+        <v>638752.20964475628</v>
       </c>
       <c r="AG43" s="7">
         <f t="shared" si="3"/>
-        <v>775692.75438316399</v>
+        <v>766889.04134576698</v>
       </c>
       <c r="AH43" s="7">
         <f t="shared" si="3"/>
-        <v>661946.98043423635</v>
+        <v>668607.96894229215</v>
       </c>
       <c r="AI43" s="7">
         <f t="shared" si="3"/>
-        <v>474092.73807401728</v>
+        <v>514361.34875161952</v>
       </c>
       <c r="AJ43" s="7">
         <f t="shared" si="3"/>
-        <v>729150.61539214232</v>
+        <v>742553.11897628871</v>
       </c>
       <c r="AK43" s="7">
         <f t="shared" si="3"/>
-        <v>903602.21151140111</v>
+        <v>893248.59419287252</v>
       </c>
       <c r="AL43" s="7">
         <f t="shared" si="3"/>
-        <v>769831.3570929959</v>
+        <v>777665.02064865385</v>
       </c>
       <c r="AM43" s="7">
         <f t="shared" si="3"/>
-        <v>548905.14916256093</v>
+        <v>596263.09723897651</v>
       </c>
       <c r="AN43" s="7">
         <f t="shared" si="3"/>
-        <v>848866.27290778619</v>
+        <v>864628.30338640453</v>
       </c>
       <c r="AO43" s="7">
         <f t="shared" si="3"/>
-        <v>1054030.2825878845</v>
+        <v>1041853.8984732302</v>
       </c>
       <c r="AP43" s="7">
         <f t="shared" si="3"/>
-        <v>896708.90817035967</v>
+        <v>905921.69762781425</v>
       </c>
       <c r="AQ43" s="7">
         <f t="shared" si="3"/>
-        <v>636888.37530781608</v>
+        <v>692583.74716865667</v>
       </c>
       <c r="AR43" s="7">
         <f t="shared" si="3"/>
-        <v>989658.01608340244</v>
+        <v>1008194.9710074639</v>
       </c>
       <c r="AS43" s="7">
         <f t="shared" si="3"/>
-        <v>1230941.3967137532</v>
+        <v>1216621.3455136498</v>
       </c>
     </row>
   </sheetData>
@@ -10143,83 +10143,83 @@
       </c>
       <c r="W2" s="4">
         <f>V2+'QTR CF'!Z43</f>
-        <v>2580327.4950840767</v>
+        <v>2585143.4922486003</v>
       </c>
       <c r="X2" s="4">
         <f>W2+'QTR CF'!AA43</f>
-        <v>2936716.4829764888</v>
+        <v>2970647.3051565615</v>
       </c>
       <c r="Y2" s="4">
         <f>X2+'QTR CF'!AB43</f>
-        <v>3477516.2400014186</v>
+        <v>3521137.2784580542</v>
       </c>
       <c r="Z2" s="4">
         <f>Y2+'QTR CF'!AC43</f>
-        <v>4144447.1847983776</v>
+        <v>4180582.3986528106</v>
       </c>
       <c r="AA2" s="4">
         <f>Z2+'QTR CF'!AD43</f>
-        <v>4714659.743908925</v>
+        <v>4756458.8170278277</v>
       </c>
       <c r="AB2" s="4">
         <f>AA2+'QTR CF'!AE43</f>
-        <v>5125139.2559386836</v>
+        <v>5201178.8540754309</v>
       </c>
       <c r="AC2" s="4">
         <f>AB2+'QTR CF'!AF43</f>
-        <v>5752495.2750630165</v>
+        <v>5839931.0637201872</v>
       </c>
       <c r="AD2" s="4">
         <f>AC2+'QTR CF'!AG43</f>
-        <v>6528188.0294461809</v>
+        <v>6606820.1050659539</v>
       </c>
       <c r="AE2" s="4">
         <f>AD2+'QTR CF'!AH43</f>
-        <v>7190135.009880417</v>
+        <v>7275428.074008246</v>
       </c>
       <c r="AF2" s="4">
         <f>AE2+'QTR CF'!AI43</f>
-        <v>7664227.7479544347</v>
+        <v>7789789.4227598654</v>
       </c>
       <c r="AG2" s="4">
         <f>AF2+'QTR CF'!AJ43</f>
-        <v>8393378.3633465767</v>
+        <v>8532342.5417361539</v>
       </c>
       <c r="AH2" s="4">
         <f>AG2+'QTR CF'!AK43</f>
-        <v>9296980.5748579782</v>
+        <v>9425591.1359290257</v>
       </c>
       <c r="AI2" s="4">
         <f>AH2+'QTR CF'!AL43</f>
-        <v>10066811.931950973</v>
+        <v>10203256.15657768</v>
       </c>
       <c r="AJ2" s="4">
         <f>AI2+'QTR CF'!AM43</f>
-        <v>10615717.081113534</v>
+        <v>10799519.253816657</v>
       </c>
       <c r="AK2" s="4">
         <f>AJ2+'QTR CF'!AN43</f>
-        <v>11464583.35402132</v>
+        <v>11664147.557203062</v>
       </c>
       <c r="AL2" s="4">
         <f>AK2+'QTR CF'!AO43</f>
-        <v>12518613.636609204</v>
+        <v>12706001.455676291</v>
       </c>
       <c r="AM2" s="4">
         <f>AL2+'QTR CF'!AP43</f>
-        <v>13415322.544779563</v>
+        <v>13611923.153304106</v>
       </c>
       <c r="AN2" s="4">
         <f>AM2+'QTR CF'!AQ43</f>
-        <v>14052210.920087378</v>
+        <v>14304506.900472762</v>
       </c>
       <c r="AO2" s="4">
         <f>AN2+'QTR CF'!AR43</f>
-        <v>15041868.936170781</v>
+        <v>15312701.871480227</v>
       </c>
       <c r="AP2" s="4">
         <f>AO2+'QTR CF'!AS43</f>
-        <v>16272810.332884535</v>
+        <v>16529323.216993876</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.25">
@@ -18327,65 +18327,85 @@
         <f>'QTR CF'!Y22</f>
         <v>-2858</v>
       </c>
-      <c r="Z22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AF22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AJ22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AK22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AL22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AM22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AN22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AO22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AP22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AQ22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AR22" s="15">
-        <v>0</v>
-      </c>
-      <c r="AS22" s="15">
-        <v>0</v>
+      <c r="Z22" s="4">
+        <f>-('QTR BS'!W14-'QTR BS'!V14)+('QTR BS'!W19-'QTR BS'!V19)+('QTR BS'!W21-'QTR BS'!V21)+('QTR BS'!W23-'QTR BS'!V23)+('QTR BS'!W25-'QTR BS'!V25)-('QTR BS'!W3-'QTR BS'!V3)-('QTR BS'!W12-'QTR BS'!V12)-('QTR BS'!W13-'QTR BS'!V13)+('QTR BS'!W24-'QTR BS'!V24)+('QTR BS'!W26-'QTR BS'!V26)+('QTR BS'!W28-'QTR BS'!V28)+('QTR BS'!W32-'QTR BS'!V32)</f>
+        <v>4815.9971645233672</v>
+      </c>
+      <c r="AA22" s="4">
+        <f>-('QTR BS'!X14-'QTR BS'!W14)+('QTR BS'!X19-'QTR BS'!W19)+('QTR BS'!X21-'QTR BS'!W21)+('QTR BS'!X23-'QTR BS'!W23)+('QTR BS'!X25-'QTR BS'!W25)-('QTR BS'!X3-'QTR BS'!W3)-('QTR BS'!X12-'QTR BS'!W12)-('QTR BS'!X13-'QTR BS'!W13)+('QTR BS'!X24-'QTR BS'!W24)+('QTR BS'!X26-'QTR BS'!W26)+('QTR BS'!X28-'QTR BS'!W28)+('QTR BS'!X32-'QTR BS'!W32)</f>
+        <v>29114.825015548769</v>
+      </c>
+      <c r="AB22" s="4">
+        <f>-('QTR BS'!Y14-'QTR BS'!X14)+('QTR BS'!Y19-'QTR BS'!X19)+('QTR BS'!Y21-'QTR BS'!X21)+('QTR BS'!Y23-'QTR BS'!X23)+('QTR BS'!Y25-'QTR BS'!X25)-('QTR BS'!Y3-'QTR BS'!X3)-('QTR BS'!Y12-'QTR BS'!X12)-('QTR BS'!Y13-'QTR BS'!X13)+('QTR BS'!Y24-'QTR BS'!X24)+('QTR BS'!Y26-'QTR BS'!X26)+('QTR BS'!Y28-'QTR BS'!X28)+('QTR BS'!Y32-'QTR BS'!X32)</f>
+        <v>9690.2162765632165</v>
+      </c>
+      <c r="AC22" s="4">
+        <f>-('QTR BS'!Z14-'QTR BS'!Y14)+('QTR BS'!Z19-'QTR BS'!Y19)+('QTR BS'!Z21-'QTR BS'!Y21)+('QTR BS'!Z23-'QTR BS'!Y23)+('QTR BS'!Z25-'QTR BS'!Y25)-('QTR BS'!Z3-'QTR BS'!Y3)-('QTR BS'!Z12-'QTR BS'!Y12)-('QTR BS'!Z13-'QTR BS'!Y13)+('QTR BS'!Z24-'QTR BS'!Y24)+('QTR BS'!Z26-'QTR BS'!Y26)+('QTR BS'!Z28-'QTR BS'!Y28)+('QTR BS'!Z32-'QTR BS'!Y32)</f>
+        <v>-7485.8246022026797</v>
+      </c>
+      <c r="AD22" s="4">
+        <f>-('QTR BS'!AA14-'QTR BS'!Z14)+('QTR BS'!AA19-'QTR BS'!Z19)+('QTR BS'!AA21-'QTR BS'!Z21)+('QTR BS'!AA23-'QTR BS'!Z23)+('QTR BS'!AA25-'QTR BS'!Z25)-('QTR BS'!AA3-'QTR BS'!Z3)-('QTR BS'!AA12-'QTR BS'!Z12)-('QTR BS'!AA13-'QTR BS'!Z13)+('QTR BS'!AA24-'QTR BS'!Z24)+('QTR BS'!AA26-'QTR BS'!Z26)+('QTR BS'!AA28-'QTR BS'!Z28)+('QTR BS'!AA32-'QTR BS'!Z32)</f>
+        <v>5663.8592644697201</v>
+      </c>
+      <c r="AE22" s="4">
+        <f>-('QTR BS'!AB14-'QTR BS'!AA14)+('QTR BS'!AB19-'QTR BS'!AA19)+('QTR BS'!AB21-'QTR BS'!AA21)+('QTR BS'!AB23-'QTR BS'!AA23)+('QTR BS'!AB25-'QTR BS'!AA25)-('QTR BS'!AB3-'QTR BS'!AA3)-('QTR BS'!AB12-'QTR BS'!AA12)-('QTR BS'!AB13-'QTR BS'!AA13)+('QTR BS'!AB24-'QTR BS'!AA24)+('QTR BS'!AB26-'QTR BS'!AA26)+('QTR BS'!AB28-'QTR BS'!AA28)+('QTR BS'!AB32-'QTR BS'!AA32)</f>
+        <v>34240.525017844666</v>
+      </c>
+      <c r="AF22" s="4">
+        <f>-('QTR BS'!AC14-'QTR BS'!AB14)+('QTR BS'!AC19-'QTR BS'!AB19)+('QTR BS'!AC21-'QTR BS'!AB21)+('QTR BS'!AC23-'QTR BS'!AB23)+('QTR BS'!AC25-'QTR BS'!AB25)-('QTR BS'!AC3-'QTR BS'!AB3)-('QTR BS'!AC12-'QTR BS'!AB12)-('QTR BS'!AC13-'QTR BS'!AB13)+('QTR BS'!AC24-'QTR BS'!AB24)+('QTR BS'!AC26-'QTR BS'!AB26)+('QTR BS'!AC28-'QTR BS'!AB28)+('QTR BS'!AC32-'QTR BS'!AB32)</f>
+        <v>11396.190520423574</v>
+      </c>
+      <c r="AG22" s="4">
+        <f>-('QTR BS'!AD14-'QTR BS'!AC14)+('QTR BS'!AD19-'QTR BS'!AC19)+('QTR BS'!AD21-'QTR BS'!AC21)+('QTR BS'!AD23-'QTR BS'!AC23)+('QTR BS'!AD25-'QTR BS'!AC25)-('QTR BS'!AD3-'QTR BS'!AC3)-('QTR BS'!AD12-'QTR BS'!AC12)-('QTR BS'!AD13-'QTR BS'!AC13)+('QTR BS'!AD24-'QTR BS'!AC24)+('QTR BS'!AD26-'QTR BS'!AC26)+('QTR BS'!AD28-'QTR BS'!AC28)+('QTR BS'!AD32-'QTR BS'!AC32)</f>
+        <v>-8803.7130373969849</v>
+      </c>
+      <c r="AH22" s="4">
+        <f>-('QTR BS'!AE14-'QTR BS'!AD14)+('QTR BS'!AE19-'QTR BS'!AD19)+('QTR BS'!AE21-'QTR BS'!AD21)+('QTR BS'!AE23-'QTR BS'!AD23)+('QTR BS'!AE25-'QTR BS'!AD25)-('QTR BS'!AE3-'QTR BS'!AD3)-('QTR BS'!AE12-'QTR BS'!AD12)-('QTR BS'!AE13-'QTR BS'!AD13)+('QTR BS'!AE24-'QTR BS'!AD24)+('QTR BS'!AE26-'QTR BS'!AD26)+('QTR BS'!AE28-'QTR BS'!AD28)+('QTR BS'!AE32-'QTR BS'!AD32)</f>
+        <v>6660.9885080558233</v>
+      </c>
+      <c r="AI22" s="4">
+        <f>-('QTR BS'!AF14-'QTR BS'!AE14)+('QTR BS'!AF19-'QTR BS'!AE19)+('QTR BS'!AF21-'QTR BS'!AE21)+('QTR BS'!AF23-'QTR BS'!AE23)+('QTR BS'!AF25-'QTR BS'!AE25)-('QTR BS'!AF3-'QTR BS'!AE3)-('QTR BS'!AF12-'QTR BS'!AE12)-('QTR BS'!AF13-'QTR BS'!AE13)+('QTR BS'!AF24-'QTR BS'!AE24)+('QTR BS'!AF26-'QTR BS'!AE26)+('QTR BS'!AF28-'QTR BS'!AE28)+('QTR BS'!AF32-'QTR BS'!AE32)</f>
+        <v>40268.610677602192</v>
+      </c>
+      <c r="AJ22" s="4">
+        <f>-('QTR BS'!AG14-'QTR BS'!AF14)+('QTR BS'!AG19-'QTR BS'!AF19)+('QTR BS'!AG21-'QTR BS'!AF21)+('QTR BS'!AG23-'QTR BS'!AF23)+('QTR BS'!AG25-'QTR BS'!AF25)-('QTR BS'!AG3-'QTR BS'!AF3)-('QTR BS'!AG12-'QTR BS'!AF12)-('QTR BS'!AG13-'QTR BS'!AF13)+('QTR BS'!AG24-'QTR BS'!AF24)+('QTR BS'!AG26-'QTR BS'!AF26)+('QTR BS'!AG28-'QTR BS'!AF28)+('QTR BS'!AG32-'QTR BS'!AF32)</f>
+        <v>13402.503584146376</v>
+      </c>
+      <c r="AK22" s="4">
+        <f>-('QTR BS'!AH14-'QTR BS'!AG14)+('QTR BS'!AH19-'QTR BS'!AG19)+('QTR BS'!AH21-'QTR BS'!AG21)+('QTR BS'!AH23-'QTR BS'!AG23)+('QTR BS'!AH25-'QTR BS'!AG25)-('QTR BS'!AH3-'QTR BS'!AG3)-('QTR BS'!AH12-'QTR BS'!AG12)-('QTR BS'!AH13-'QTR BS'!AG13)+('QTR BS'!AH24-'QTR BS'!AG24)+('QTR BS'!AH26-'QTR BS'!AG26)+('QTR BS'!AH28-'QTR BS'!AG28)+('QTR BS'!AH32-'QTR BS'!AG32)</f>
+        <v>-10353.617318528588</v>
+      </c>
+      <c r="AL22" s="4">
+        <f>-('QTR BS'!AI14-'QTR BS'!AH14)+('QTR BS'!AI19-'QTR BS'!AH19)+('QTR BS'!AI21-'QTR BS'!AH21)+('QTR BS'!AI23-'QTR BS'!AH23)+('QTR BS'!AI25-'QTR BS'!AH25)-('QTR BS'!AI3-'QTR BS'!AH3)-('QTR BS'!AI12-'QTR BS'!AH12)-('QTR BS'!AI13-'QTR BS'!AH13)+('QTR BS'!AI24-'QTR BS'!AH24)+('QTR BS'!AI26-'QTR BS'!AH26)+('QTR BS'!AI28-'QTR BS'!AH28)+('QTR BS'!AI32-'QTR BS'!AH32)</f>
+        <v>7833.6635556578985</v>
+      </c>
+      <c r="AM22" s="4">
+        <f>-('QTR BS'!AJ14-'QTR BS'!AI14)+('QTR BS'!AJ19-'QTR BS'!AI19)+('QTR BS'!AJ21-'QTR BS'!AI21)+('QTR BS'!AJ23-'QTR BS'!AI23)+('QTR BS'!AJ25-'QTR BS'!AI25)-('QTR BS'!AJ3-'QTR BS'!AI3)-('QTR BS'!AJ12-'QTR BS'!AI12)-('QTR BS'!AJ13-'QTR BS'!AI13)+('QTR BS'!AJ24-'QTR BS'!AI24)+('QTR BS'!AJ26-'QTR BS'!AI26)+('QTR BS'!AJ28-'QTR BS'!AI28)+('QTR BS'!AJ32-'QTR BS'!AI32)</f>
+        <v>47357.948076415589</v>
+      </c>
+      <c r="AN22" s="4">
+        <f>-('QTR BS'!AK14-'QTR BS'!AJ14)+('QTR BS'!AK19-'QTR BS'!AJ19)+('QTR BS'!AK21-'QTR BS'!AJ21)+('QTR BS'!AK23-'QTR BS'!AJ23)+('QTR BS'!AK25-'QTR BS'!AJ25)-('QTR BS'!AK3-'QTR BS'!AJ3)-('QTR BS'!AK12-'QTR BS'!AJ12)-('QTR BS'!AK13-'QTR BS'!AJ13)+('QTR BS'!AK24-'QTR BS'!AJ24)+('QTR BS'!AK26-'QTR BS'!AJ26)+('QTR BS'!AK28-'QTR BS'!AJ28)+('QTR BS'!AK32-'QTR BS'!AJ32)</f>
+        <v>15762.030478618326</v>
+      </c>
+      <c r="AO22" s="4">
+        <f>-('QTR BS'!AL14-'QTR BS'!AK14)+('QTR BS'!AL19-'QTR BS'!AK19)+('QTR BS'!AL21-'QTR BS'!AK21)+('QTR BS'!AL23-'QTR BS'!AK23)+('QTR BS'!AL25-'QTR BS'!AK25)-('QTR BS'!AL3-'QTR BS'!AK3)-('QTR BS'!AL12-'QTR BS'!AK12)-('QTR BS'!AL13-'QTR BS'!AK13)+('QTR BS'!AL24-'QTR BS'!AK24)+('QTR BS'!AL26-'QTR BS'!AK26)+('QTR BS'!AL28-'QTR BS'!AK28)+('QTR BS'!AL32-'QTR BS'!AK32)</f>
+        <v>-12176.384114654415</v>
+      </c>
+      <c r="AP22" s="4">
+        <f>-('QTR BS'!AM14-'QTR BS'!AL14)+('QTR BS'!AM19-'QTR BS'!AL19)+('QTR BS'!AM21-'QTR BS'!AL21)+('QTR BS'!AM23-'QTR BS'!AL23)+('QTR BS'!AM25-'QTR BS'!AL25)-('QTR BS'!AM3-'QTR BS'!AL3)-('QTR BS'!AM12-'QTR BS'!AL12)-('QTR BS'!AM13-'QTR BS'!AL13)+('QTR BS'!AM24-'QTR BS'!AL24)+('QTR BS'!AM26-'QTR BS'!AL26)+('QTR BS'!AM28-'QTR BS'!AL28)+('QTR BS'!AM32-'QTR BS'!AL32)</f>
+        <v>9212.7894574545571</v>
+      </c>
+      <c r="AQ22" s="4">
+        <f>-('QTR BS'!AN14-'QTR BS'!AM14)+('QTR BS'!AN19-'QTR BS'!AM19)+('QTR BS'!AN21-'QTR BS'!AM21)+('QTR BS'!AN23-'QTR BS'!AM23)+('QTR BS'!AN25-'QTR BS'!AM25)-('QTR BS'!AN3-'QTR BS'!AM3)-('QTR BS'!AN12-'QTR BS'!AM12)-('QTR BS'!AN13-'QTR BS'!AM13)+('QTR BS'!AN24-'QTR BS'!AM24)+('QTR BS'!AN26-'QTR BS'!AM26)+('QTR BS'!AN28-'QTR BS'!AM28)+('QTR BS'!AN32-'QTR BS'!AM32)</f>
+        <v>55695.371860840714</v>
+      </c>
+      <c r="AR22" s="4">
+        <f>-('QTR BS'!AO14-'QTR BS'!AN14)+('QTR BS'!AO19-'QTR BS'!AN19)+('QTR BS'!AO21-'QTR BS'!AN21)+('QTR BS'!AO23-'QTR BS'!AN23)+('QTR BS'!AO25-'QTR BS'!AN25)-('QTR BS'!AO3-'QTR BS'!AN3)-('QTR BS'!AO12-'QTR BS'!AN12)-('QTR BS'!AO13-'QTR BS'!AN13)+('QTR BS'!AO24-'QTR BS'!AN24)+('QTR BS'!AO26-'QTR BS'!AN26)+('QTR BS'!AO28-'QTR BS'!AN28)+('QTR BS'!AO32-'QTR BS'!AN32)</f>
+        <v>18536.954924061356</v>
+      </c>
+      <c r="AS22" s="4">
+        <f>-('QTR BS'!AP14-'QTR BS'!AO14)+('QTR BS'!AP19-'QTR BS'!AO19)+('QTR BS'!AP21-'QTR BS'!AO21)+('QTR BS'!AP23-'QTR BS'!AO23)+('QTR BS'!AP25-'QTR BS'!AO25)-('QTR BS'!AP3-'QTR BS'!AO3)-('QTR BS'!AP12-'QTR BS'!AO12)-('QTR BS'!AP13-'QTR BS'!AO13)+('QTR BS'!AP24-'QTR BS'!AO24)+('QTR BS'!AP26-'QTR BS'!AO26)+('QTR BS'!AP28-'QTR BS'!AO28)+('QTR BS'!AP32-'QTR BS'!AO32)</f>
+        <v>-14320.051200103422</v>
       </c>
     </row>
     <row r="23" spans="1:45" x14ac:dyDescent="0.25">
@@ -22013,23 +22033,23 @@
       </c>
       <c r="H2" s="11">
         <f>'QTR BS'!Z2</f>
-        <v>4144447.1847983776</v>
+        <v>4180582.3986528106</v>
       </c>
       <c r="I2" s="11">
         <f>'QTR BS'!AD2</f>
-        <v>6528188.0294461809</v>
+        <v>6606820.1050659539</v>
       </c>
       <c r="J2" s="11">
         <f>'QTR BS'!AH2</f>
-        <v>9296980.5748579782</v>
+        <v>9425591.1359290257</v>
       </c>
       <c r="K2" s="11">
         <f>'QTR BS'!AL2</f>
-        <v>12518613.636609204</v>
+        <v>12706001.455676291</v>
       </c>
       <c r="L2" s="11">
         <f>'QTR BS'!AP2</f>
-        <v>16272810.332884535</v>
+        <v>16529323.216993876</v>
       </c>
       <c r="M2" s="5"/>
     </row>
@@ -22283,23 +22303,23 @@
       </c>
       <c r="H8" s="7">
         <f t="shared" si="0"/>
-        <v>7874422.5127534289</v>
+        <v>7910557.7266078629</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" si="0"/>
-        <v>10795628.551794514</v>
+        <v>10874260.627414286</v>
       </c>
       <c r="J8" s="7">
         <f t="shared" si="0"/>
-        <v>14196507.686255559</v>
+        <v>14325118.247326607</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
-        <v>18161506.942178532</v>
+        <v>18348894.76124562</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" si="0"/>
-        <v>22789940.346226081</v>
+        <v>23046453.230335422</v>
       </c>
       <c r="M8" s="7">
         <f t="shared" si="0"/>
@@ -22600,23 +22620,23 @@
       </c>
       <c r="H15" s="7">
         <f t="shared" si="1"/>
-        <v>12581700.122867659</v>
+        <v>12617835.336722095</v>
       </c>
       <c r="I15" s="7">
         <f t="shared" si="1"/>
-        <v>15598948.450948428</v>
+        <v>15677580.5265682</v>
       </c>
       <c r="J15" s="7">
         <f t="shared" si="1"/>
-        <v>19115422.52416908</v>
+        <v>19244033.085240126</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>23219011.636098877</v>
+        <v>23406399.455165967</v>
       </c>
       <c r="L15" s="7">
         <f t="shared" si="1"/>
-        <v>28013078.096270941</v>
+        <v>28269590.980380282</v>
       </c>
       <c r="M15" s="7">
         <f t="shared" si="1"/>
@@ -24380,23 +24400,23 @@
       </c>
       <c r="I20" s="11">
         <f>'QTR CF'!Z22+'QTR CF'!AA22+'QTR CF'!AB22+'QTR CF'!AC22</f>
-        <v>0</v>
+        <v>36135.213854432674</v>
       </c>
       <c r="J20" s="11">
         <f>'QTR CF'!AD22+'QTR CF'!AE22+'QTR CF'!AF22+'QTR CF'!AG22</f>
-        <v>0</v>
+        <v>42496.861765340975</v>
       </c>
       <c r="K20" s="11">
         <f>'QTR CF'!AH22+'QTR CF'!AI22+'QTR CF'!AJ22+'QTR CF'!AK22</f>
-        <v>0</v>
+        <v>49978.485451275803</v>
       </c>
       <c r="L20" s="11">
         <f>'QTR CF'!AL22+'QTR CF'!AM22+'QTR CF'!AN22+'QTR CF'!AO22</f>
-        <v>0</v>
+        <v>58777.257996037399</v>
       </c>
       <c r="M20" s="11">
         <f>'QTR CF'!AP22+'QTR CF'!AQ22+'QTR CF'!AR22+'QTR CF'!AS22</f>
-        <v>0</v>
+        <v>69125.065042253205</v>
       </c>
       <c r="N20" s="5"/>
     </row>
@@ -24481,23 +24501,23 @@
       </c>
       <c r="I22" s="7">
         <f t="shared" si="0"/>
-        <v>2170631.2563160751</v>
+        <v>2206766.4701705077</v>
       </c>
       <c r="J22" s="7">
         <f t="shared" si="0"/>
-        <v>2535850.1572036459</v>
+        <v>2578347.0189689868</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="0"/>
-        <v>2965366.2853669473</v>
+        <v>3015344.7708182232</v>
       </c>
       <c r="L22" s="7">
         <f t="shared" si="0"/>
-        <v>3470499.2450907002</v>
+        <v>3529276.5030867378</v>
       </c>
       <c r="M22" s="7">
         <f t="shared" si="0"/>
-        <v>4064561.4706243305</v>
+        <v>4133686.5356665836</v>
       </c>
       <c r="N22" s="7">
         <f t="shared" si="0"/>
@@ -25357,23 +25377,23 @@
       </c>
       <c r="I40" s="7">
         <f t="shared" si="3"/>
-        <v>2056330.1847983776</v>
+        <v>2092465.3986528101</v>
       </c>
       <c r="J40" s="7">
         <f t="shared" si="3"/>
-        <v>2383740.8446478024</v>
+        <v>2426237.7064131433</v>
       </c>
       <c r="K40" s="7">
         <f t="shared" si="3"/>
-        <v>2768792.5454117982</v>
+        <v>2818771.0308630741</v>
       </c>
       <c r="L40" s="7">
         <f t="shared" si="3"/>
-        <v>3221633.0617512278</v>
+        <v>3280410.3197472654</v>
       </c>
       <c r="M40" s="7">
         <f t="shared" si="3"/>
-        <v>3754196.6962753325</v>
+        <v>3823321.7613175856</v>
       </c>
       <c r="N40" s="7">
         <f t="shared" si="3"/>
@@ -33799,83 +33819,83 @@
       </c>
       <c r="W2" s="11">
         <f>'BS DRIVERS'!W2</f>
-        <v>2580327.4950840767</v>
+        <v>2585143.4922486003</v>
       </c>
       <c r="X2" s="11">
         <f>'BS DRIVERS'!X2</f>
-        <v>2936716.4829764888</v>
+        <v>2970647.3051565615</v>
       </c>
       <c r="Y2" s="11">
         <f>'BS DRIVERS'!Y2</f>
-        <v>3477516.2400014186</v>
+        <v>3521137.2784580542</v>
       </c>
       <c r="Z2" s="11">
         <f>'BS DRIVERS'!Z2</f>
-        <v>4144447.1847983776</v>
+        <v>4180582.3986528106</v>
       </c>
       <c r="AA2" s="11">
         <f>'BS DRIVERS'!AA2</f>
-        <v>4714659.743908925</v>
+        <v>4756458.8170278277</v>
       </c>
       <c r="AB2" s="11">
         <f>'BS DRIVERS'!AB2</f>
-        <v>5125139.2559386836</v>
+        <v>5201178.8540754309</v>
       </c>
       <c r="AC2" s="11">
         <f>'BS DRIVERS'!AC2</f>
-        <v>5752495.2750630165</v>
+        <v>5839931.0637201872</v>
       </c>
       <c r="AD2" s="11">
         <f>'BS DRIVERS'!AD2</f>
-        <v>6528188.0294461809</v>
+        <v>6606820.1050659539</v>
       </c>
       <c r="AE2" s="11">
         <f>'BS DRIVERS'!AE2</f>
-        <v>7190135.009880417</v>
+        <v>7275428.074008246</v>
       </c>
       <c r="AF2" s="11">
         <f>'BS DRIVERS'!AF2</f>
-        <v>7664227.7479544347</v>
+        <v>7789789.4227598654</v>
       </c>
       <c r="AG2" s="11">
         <f>'BS DRIVERS'!AG2</f>
-        <v>8393378.3633465767</v>
+        <v>8532342.5417361539</v>
       </c>
       <c r="AH2" s="11">
         <f>'BS DRIVERS'!AH2</f>
-        <v>9296980.5748579782</v>
+        <v>9425591.1359290257</v>
       </c>
       <c r="AI2" s="11">
         <f>'BS DRIVERS'!AI2</f>
-        <v>10066811.931950973</v>
+        <v>10203256.15657768</v>
       </c>
       <c r="AJ2" s="11">
         <f>'BS DRIVERS'!AJ2</f>
-        <v>10615717.081113534</v>
+        <v>10799519.253816657</v>
       </c>
       <c r="AK2" s="11">
         <f>'BS DRIVERS'!AK2</f>
-        <v>11464583.35402132</v>
+        <v>11664147.557203062</v>
       </c>
       <c r="AL2" s="11">
         <f>'BS DRIVERS'!AL2</f>
-        <v>12518613.636609204</v>
+        <v>12706001.455676291</v>
       </c>
       <c r="AM2" s="11">
         <f>'BS DRIVERS'!AM2</f>
-        <v>13415322.544779563</v>
+        <v>13611923.153304106</v>
       </c>
       <c r="AN2" s="11">
         <f>'BS DRIVERS'!AN2</f>
-        <v>14052210.920087378</v>
+        <v>14304506.900472762</v>
       </c>
       <c r="AO2" s="11">
         <f>'BS DRIVERS'!AO2</f>
-        <v>15041868.936170781</v>
+        <v>15312701.871480227</v>
       </c>
       <c r="AP2" s="11">
         <f>'BS DRIVERS'!AP2</f>
-        <v>16272810.332884535</v>
+        <v>16529323.216993876</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.25">
@@ -34813,83 +34833,83 @@
       </c>
       <c r="W8" s="7">
         <f t="shared" ref="W8:AP8" si="0">SUM(W2:W7)</f>
-        <v>5914203.2479826044</v>
+        <v>5919019.2451471277</v>
       </c>
       <c r="X8" s="7">
         <f t="shared" si="0"/>
-        <v>6638812.4864223273</v>
+        <v>6672743.3086024001</v>
       </c>
       <c r="Y8" s="7">
         <f t="shared" si="0"/>
-        <v>7302166.0923303673</v>
+        <v>7345787.1307870029</v>
       </c>
       <c r="Z8" s="7">
         <f t="shared" si="0"/>
-        <v>7874422.5127534289</v>
+        <v>7910557.7266078629</v>
       </c>
       <c r="AA8" s="7">
         <f t="shared" si="0"/>
-        <v>8516266.8840529192</v>
+        <v>8558065.957171822</v>
       </c>
       <c r="AB8" s="7">
         <f t="shared" si="0"/>
-        <v>9359792.2651273627</v>
+        <v>9435831.8632641099</v>
       </c>
       <c r="AC8" s="7">
         <f t="shared" si="0"/>
-        <v>10131277.885802597</v>
+        <v>10218713.674459768</v>
       </c>
       <c r="AD8" s="7">
         <f t="shared" si="0"/>
-        <v>10795628.551794514</v>
+        <v>10874260.627414286</v>
       </c>
       <c r="AE8" s="7">
         <f t="shared" si="0"/>
-        <v>11541818.211208247</v>
+        <v>11627111.275336076</v>
       </c>
       <c r="AF8" s="7">
         <f t="shared" si="0"/>
-        <v>12525195.065019868</v>
+        <v>12650756.739825297</v>
       </c>
       <c r="AG8" s="7">
         <f t="shared" si="0"/>
-        <v>13423849.471868083</v>
+        <v>13562813.65025766</v>
       </c>
       <c r="AH8" s="7">
         <f t="shared" si="0"/>
-        <v>14196507.686255559</v>
+        <v>14325118.247326607</v>
       </c>
       <c r="AI8" s="7">
         <f t="shared" si="0"/>
-        <v>15065412.74740232</v>
+        <v>15201856.972029027</v>
       </c>
       <c r="AJ8" s="7">
         <f t="shared" si="0"/>
-        <v>16213262.094127169</v>
+        <v>16397064.266830293</v>
       </c>
       <c r="AK8" s="7">
         <f t="shared" si="0"/>
-        <v>17261473.505083065</v>
+        <v>17461037.708264805</v>
       </c>
       <c r="AL8" s="7">
         <f t="shared" si="0"/>
-        <v>18161506.942178532</v>
+        <v>18348894.76124562</v>
       </c>
       <c r="AM8" s="7">
         <f t="shared" si="0"/>
-        <v>19174731.599299874</v>
+        <v>19371332.207824416</v>
       </c>
       <c r="AN8" s="7">
         <f t="shared" si="0"/>
-        <v>20516009.019363139</v>
+        <v>20768304.999748524</v>
       </c>
       <c r="AO8" s="7">
         <f t="shared" si="0"/>
-        <v>21740107.125087362</v>
+        <v>22010940.060396809</v>
       </c>
       <c r="AP8" s="7">
         <f t="shared" si="0"/>
-        <v>22789940.346226081</v>
+        <v>23046453.230335422</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.25">
@@ -35996,83 +36016,83 @@
       </c>
       <c r="W15" s="7">
         <f t="shared" ref="W15:AP15" si="1">W8+SUM(W9:W14)</f>
-        <v>10549140.984553687</v>
+        <v>10553956.981718209</v>
       </c>
       <c r="X15" s="7">
         <f t="shared" si="1"/>
-        <v>11356791.114141569</v>
+        <v>11390721.936321642</v>
       </c>
       <c r="Y15" s="7">
         <f t="shared" si="1"/>
-        <v>12041777.866520908</v>
+        <v>12085398.904977543</v>
       </c>
       <c r="Z15" s="7">
         <f t="shared" si="1"/>
-        <v>12581700.122867659</v>
+        <v>12617835.336722095</v>
       </c>
       <c r="AA15" s="7">
         <f t="shared" si="1"/>
-        <v>13232528.171004493</v>
+        <v>13274327.244123396</v>
       </c>
       <c r="AB15" s="7">
         <f t="shared" si="1"/>
-        <v>14174374.964378081</v>
+        <v>14250414.562514829</v>
       </c>
       <c r="AC15" s="7">
         <f t="shared" si="1"/>
-        <v>14971963.345281754</v>
+        <v>15059399.133938927</v>
       </c>
       <c r="AD15" s="7">
         <f t="shared" si="1"/>
-        <v>15598948.450948428</v>
+        <v>15677580.5265682</v>
       </c>
       <c r="AE15" s="7">
         <f t="shared" si="1"/>
-        <v>16356364.446595863</v>
+        <v>16441657.510723691</v>
       </c>
       <c r="AF15" s="7">
         <f t="shared" si="1"/>
-        <v>17456033.388006125</v>
+        <v>17581595.062811553</v>
       </c>
       <c r="AG15" s="7">
         <f t="shared" si="1"/>
-        <v>18386047.049723901</v>
+        <v>18525011.22811348</v>
       </c>
       <c r="AH15" s="7">
         <f t="shared" si="1"/>
-        <v>19115422.52416908</v>
+        <v>19244033.085240126</v>
       </c>
       <c r="AI15" s="7">
         <f t="shared" si="1"/>
-        <v>19998191.403833099</v>
+        <v>20134635.628459804</v>
       </c>
       <c r="AJ15" s="7">
         <f t="shared" si="1"/>
-        <v>21283467.272481762</v>
+        <v>21467269.445184886</v>
       </c>
       <c r="AK15" s="7">
         <f t="shared" si="1"/>
-        <v>22369219.845159464</v>
+        <v>22568784.048341203</v>
       </c>
       <c r="AL15" s="7">
         <f t="shared" si="1"/>
-        <v>23219011.636098877</v>
+        <v>23406399.455165967</v>
       </c>
       <c r="AM15" s="7">
         <f t="shared" si="1"/>
-        <v>24249201.925952956</v>
+        <v>24445802.534477498</v>
       </c>
       <c r="AN15" s="7">
         <f t="shared" si="1"/>
-        <v>25752761.044876959</v>
+        <v>26005057.025262345</v>
       </c>
       <c r="AO15" s="7">
         <f t="shared" si="1"/>
-        <v>27021670.551320449</v>
+        <v>27292503.486629896</v>
       </c>
       <c r="AP15" s="7">
         <f t="shared" si="1"/>
-        <v>28013078.096270941</v>
+        <v>28269590.980380282</v>
       </c>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.25">

</xml_diff>